<commit_message>
BRD-13 Data Migration screenshots retaken in the BDO style-guide presentation on a fresh seed stack: 71 images; Handbook, guide deck, migration workbook and UX documents 07 to 09 rebuilt at v2.0 with issue 2.2 change CHG-DM-2.2-01; Remove of a legacy batch line described in its row action menu; drop indexes
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-13_Data_Migration/08_BIBS_UXScreens_BRD-13_Data_Migration_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-13_Data_Migration/08_BIBS_UXScreens_BRD-13_Data_Migration_v2.0.xlsx
@@ -689,7 +689,7 @@
 Mandatory: Yes
 Format: Y or N
 Allowed values: Y or N
-Example: N</t>
+Example: Y</t>
       </text>
     </comment>
     <comment ref="O16" authorId="0" shapeId="0">
@@ -698,7 +698,8 @@
 The change reference (comment, change request or issue change) that changed the image
 Mandatory: Conditional: when Changed in this issue is Y
 Format: Reference
-Allowed values: Free entry</t>
+Allowed values: Free entry
+Example: CHG-DM-2.2-01</t>
       </text>
     </comment>
   </commentList>
@@ -1073,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:I37"/>
+  <dimension ref="A2:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1348,7 +1349,7 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>75 screen images of 35 screens; 15 changed in this issue</t>
+          <t>75 screen images of 35 screens; 57 changed in this issue</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
@@ -1520,43 +1521,47 @@
       </c>
       <c r="I30" s="5" t="n"/>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Lists in the BDO style guide: outlined status pills, alternating white and Background Blue rows, a long list scrolling inside its card with the header row in view, names instead of codes, due dates on one line with the overdue icon and ages in words; every image of the set retaken</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>SCR-DM-01, SCR-DM-02, SCR-DM-03, SCR-DM-04, SCR-DM-05, SCR-DM-06, SCR-DM-07, SCR-DM-08, SCR-DM-09, SCR-DM-10, SCR-DM-11, SCR-DM-12, SCR-DM-13, SCR-DM-14, SCR-DM-15, SCR-DM-16, SCR-DM-17, SCR-DM-18, SCR-DM-19, SCR-DM-20</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Other sheets</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Sheet</t>
-        </is>
-      </c>
-      <c r="B33" s="18" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>What it holds</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="5" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Reference lists</t>
         </is>
       </c>
       <c r="B34" s="18" t="n"/>
       <c r="C34" s="5" t="n"/>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>The lists of the drop-downs: states and UXD statuses</t>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>What it holds</t>
         </is>
       </c>
       <c r="E34" s="18" t="n"/>
@@ -1568,14 +1573,14 @@
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Questions and comments</t>
+          <t>Reference lists</t>
         </is>
       </c>
       <c r="B35" s="18" t="n"/>
       <c r="C35" s="5" t="n"/>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>Questions and comments of the UX Design team, with the answer</t>
+          <t>The lists of the drop-downs: states and UXD statuses</t>
         </is>
       </c>
       <c r="E35" s="18" t="n"/>
@@ -1584,8 +1589,27 @@
       <c r="H35" s="18" t="n"/>
       <c r="I35" s="5" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Questions and comments</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Questions and comments of the UX Design team, with the answer</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="n"/>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Prepared by iorta TechNXT for BDOI. Confidential – BDOI.</t>
         </is>
@@ -1593,7 +1617,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A21:I22"/>
-  <mergeCells count="41">
+  <mergeCells count="44">
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="C30:G30"/>
@@ -1601,23 +1625,23 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C9:H9"/>
     <mergeCell ref="B16:I16"/>
+    <mergeCell ref="H31:I31"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C26:G26"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="C11:H11"/>
     <mergeCell ref="H25:I25"/>
     <mergeCell ref="C29:G29"/>
-    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C25:G25"/>
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C31:G31"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="B17:I17"/>
-    <mergeCell ref="D33:I33"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="C27:G27"/>
     <mergeCell ref="D35:I35"/>
@@ -1627,12 +1651,15 @@
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="D34:I34"/>
     <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="B15:I15"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:G28"/>
+    <mergeCell ref="D36:I36"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A31:B31"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="H26:I26"/>
   </mergeCells>
@@ -1662,8 +1689,8 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="I22" location="'UX screen register'!A1"/>
-    <hyperlink ref="A34" location="'Reference lists'!A1"/>
-    <hyperlink ref="A35" location="'Questions and comments'!A1"/>
+    <hyperlink ref="A35" location="'Reference lists'!A1"/>
+    <hyperlink ref="A36" location="'Questions and comments'!A1"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
@@ -2306,10 +2333,14 @@
       <c r="M17" s="43" t="n"/>
       <c r="N17" s="43" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O17" s="43" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O17" s="43" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="45" t="inlineStr">
@@ -2366,10 +2397,14 @@
       <c r="M18" s="45" t="n"/>
       <c r="N18" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O18" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O18" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="45" t="inlineStr">
@@ -2428,10 +2463,14 @@
       <c r="M19" s="45" t="n"/>
       <c r="N19" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O19" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O19" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="45" t="inlineStr">
@@ -2490,10 +2529,14 @@
       <c r="M20" s="45" t="n"/>
       <c r="N20" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O20" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O20" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="45" t="inlineStr">
@@ -2550,10 +2593,14 @@
       <c r="M21" s="45" t="n"/>
       <c r="N21" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O21" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O21" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="45" t="inlineStr">
@@ -2610,10 +2657,14 @@
       <c r="M22" s="45" t="n"/>
       <c r="N22" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O22" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O22" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="45" t="inlineStr">
@@ -2672,10 +2723,14 @@
       <c r="M23" s="45" t="n"/>
       <c r="N23" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O23" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O23" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="45" t="inlineStr">
@@ -2734,10 +2789,14 @@
       <c r="M24" s="45" t="n"/>
       <c r="N24" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O24" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O24" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="45" t="inlineStr">
@@ -2794,10 +2853,14 @@
       <c r="M25" s="45" t="n"/>
       <c r="N25" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O25" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O25" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="45" t="inlineStr">
@@ -2854,10 +2917,14 @@
       <c r="M26" s="45" t="n"/>
       <c r="N26" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O26" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O26" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="45" t="inlineStr">
@@ -2914,10 +2981,14 @@
       <c r="M27" s="45" t="n"/>
       <c r="N27" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O27" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O27" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="45" t="inlineStr">
@@ -2974,10 +3045,14 @@
       <c r="M28" s="45" t="n"/>
       <c r="N28" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O28" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O28" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="45" t="inlineStr">
@@ -3041,7 +3116,7 @@
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
-          <t>CHG-DM-2.1-02, CHG-DM-2.1-03, CHG-DM-2.1-04</t>
+          <t>CHG-DM-2.1-02, CHG-DM-2.1-03, CHG-DM-2.1-04, CHG-DM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3182,7 @@
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
-          <t>CHG-DM-2.1-03, CHG-DM-2.1-04</t>
+          <t>CHG-DM-2.1-03, CHG-DM-2.1-04, CHG-DM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3166,10 +3241,14 @@
       <c r="M31" s="45" t="n"/>
       <c r="N31" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O31" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O31" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="45" t="inlineStr">
@@ -3228,10 +3307,14 @@
       <c r="M32" s="45" t="n"/>
       <c r="N32" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O32" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O32" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="45" t="inlineStr">
@@ -3288,10 +3371,14 @@
       <c r="M33" s="45" t="n"/>
       <c r="N33" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O33" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O33" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="45" t="inlineStr">
@@ -3350,10 +3437,14 @@
       <c r="M34" s="45" t="n"/>
       <c r="N34" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O34" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O34" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="45" t="inlineStr">
@@ -3410,10 +3501,14 @@
       <c r="M35" s="45" t="n"/>
       <c r="N35" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O35" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O35" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="45" t="inlineStr">
@@ -3472,10 +3567,14 @@
       <c r="M36" s="45" t="n"/>
       <c r="N36" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O36" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O36" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="45" t="inlineStr">
@@ -3534,10 +3633,14 @@
       <c r="M37" s="45" t="n"/>
       <c r="N37" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O37" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O37" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="45" t="inlineStr">
@@ -3594,10 +3697,14 @@
       <c r="M38" s="45" t="n"/>
       <c r="N38" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O38" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O38" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="45" t="inlineStr">
@@ -3654,10 +3761,14 @@
       <c r="M39" s="45" t="n"/>
       <c r="N39" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O39" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O39" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="45" t="inlineStr">
@@ -3716,10 +3827,14 @@
       <c r="M40" s="45" t="n"/>
       <c r="N40" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O40" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O40" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="45" t="inlineStr">
@@ -3778,10 +3893,14 @@
       <c r="M41" s="45" t="n"/>
       <c r="N41" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O41" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O41" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="45" t="inlineStr">
@@ -3840,10 +3959,14 @@
       <c r="M42" s="45" t="n"/>
       <c r="N42" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O42" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O42" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="45" t="inlineStr">
@@ -3902,10 +4025,14 @@
       <c r="M43" s="45" t="n"/>
       <c r="N43" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O43" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O43" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="45" t="inlineStr">
@@ -3964,10 +4091,14 @@
       <c r="M44" s="45" t="n"/>
       <c r="N44" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O44" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O44" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="45" t="inlineStr">
@@ -4026,10 +4157,14 @@
       <c r="M45" s="45" t="n"/>
       <c r="N45" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O45" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O45" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="45" t="inlineStr">
@@ -4088,10 +4223,14 @@
       <c r="M46" s="45" t="n"/>
       <c r="N46" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O46" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O46" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="45" t="inlineStr">
@@ -4150,10 +4289,14 @@
       <c r="M47" s="45" t="n"/>
       <c r="N47" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O47" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O47" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="45" t="inlineStr">
@@ -4217,7 +4360,7 @@
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
-          <t>CHG-DM-2.1-02</t>
+          <t>CHG-DM-2.1-02, CHG-DM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -4278,10 +4421,14 @@
       <c r="M49" s="45" t="n"/>
       <c r="N49" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O49" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O49" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="45" t="inlineStr">
@@ -4340,10 +4487,14 @@
       <c r="M50" s="45" t="n"/>
       <c r="N50" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O50" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O50" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="45" t="inlineStr">
@@ -4402,10 +4553,14 @@
       <c r="M51" s="45" t="n"/>
       <c r="N51" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O51" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O51" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="45" t="inlineStr">
@@ -4464,10 +4619,14 @@
       <c r="M52" s="45" t="n"/>
       <c r="N52" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O52" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O52" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="45" t="inlineStr">
@@ -4526,10 +4685,14 @@
       <c r="M53" s="45" t="n"/>
       <c r="N53" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O53" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O53" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="45" t="inlineStr">
@@ -4588,10 +4751,14 @@
       <c r="M54" s="45" t="n"/>
       <c r="N54" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O54" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O54" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="45" t="inlineStr">
@@ -4650,10 +4817,14 @@
       <c r="M55" s="45" t="n"/>
       <c r="N55" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O55" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O55" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="45" t="inlineStr">
@@ -4712,10 +4883,14 @@
       <c r="M56" s="45" t="n"/>
       <c r="N56" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O56" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O56" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="45" t="inlineStr">
@@ -4772,10 +4947,14 @@
       <c r="M57" s="45" t="n"/>
       <c r="N57" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O57" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O57" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="45" t="inlineStr">
@@ -4834,10 +5013,14 @@
       <c r="M58" s="45" t="n"/>
       <c r="N58" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O58" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O58" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="45" t="inlineStr">
@@ -4896,10 +5079,14 @@
       <c r="M59" s="45" t="n"/>
       <c r="N59" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O59" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O59" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="45" t="inlineStr">
@@ -4958,10 +5145,14 @@
       <c r="M60" s="45" t="n"/>
       <c r="N60" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O60" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O60" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="45" t="inlineStr">
@@ -5020,10 +5211,14 @@
       <c r="M61" s="45" t="n"/>
       <c r="N61" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O61" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O61" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="45" t="inlineStr">
@@ -6928,10 +7123,14 @@
       <c r="M92" s="45" t="n"/>
       <c r="N92" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O92" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O92" s="45" t="inlineStr">
+        <is>
+          <t>CHG-DM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="46" t="n"/>

</xml_diff>